<commit_message>
Updated TD average and added TD individuals with notes.
</commit_message>
<xml_diff>
--- a/data/aperiodic.xlsx
+++ b/data/aperiodic.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1276,64 +1276,64 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.057093547330473</v>
+        <v>2.024668147718512</v>
       </c>
       <c r="D12" t="n">
-        <v>1.959760537708682</v>
+        <v>1.96868605083528</v>
       </c>
       <c r="E12" t="n">
-        <v>2.018522577006388</v>
+        <v>1.997235502033564</v>
       </c>
       <c r="F12" t="n">
-        <v>1.843825449929359</v>
+        <v>1.890965750974551</v>
       </c>
       <c r="G12" t="n">
-        <v>1.986383989072011</v>
+        <v>1.973309945131826</v>
       </c>
       <c r="H12" t="n">
-        <v>1.979454547823752</v>
+        <v>2.025951767250887</v>
       </c>
       <c r="I12" t="n">
-        <v>1.757312822854038</v>
+        <v>1.834479080590469</v>
       </c>
       <c r="J12" t="n">
-        <v>2.145466290143831</v>
+        <v>2.175618676112611</v>
       </c>
       <c r="K12" t="n">
-        <v>1.929526700683982</v>
+        <v>1.991936647761554</v>
       </c>
       <c r="L12" t="n">
-        <v>1.821971139194069</v>
+        <v>1.836382690079349</v>
       </c>
       <c r="M12" t="n">
         <v>1.995904382483224</v>
       </c>
       <c r="N12" t="n">
-        <v>2.369037164018575</v>
+        <v>2.348177949782953</v>
       </c>
       <c r="O12" t="n">
-        <v>2.448812293885807</v>
+        <v>2.415581819369827</v>
       </c>
       <c r="P12" t="n">
-        <v>2.211831315665458</v>
+        <v>2.222630520845329</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.085934481024001</v>
+        <v>2.104067893024136</v>
       </c>
       <c r="R12" t="n">
-        <v>2.138946561132661</v>
+        <v>2.103428264261743</v>
       </c>
       <c r="S12" t="n">
-        <v>1.672039069492139</v>
+        <v>1.694906160218784</v>
       </c>
       <c r="T12" t="n">
-        <v>1.441563175449537</v>
+        <v>1.566122955680536</v>
       </c>
       <c r="U12" t="n">
-        <v>2.327030767708496</v>
+        <v>2.33547336142582</v>
       </c>
       <c r="V12" t="n">
-        <v>2.137540924940734</v>
+        <v>2.160336426143453</v>
       </c>
     </row>
     <row r="13">
@@ -3278,6 +3278,726 @@
       </c>
       <c r="V39" t="n">
         <v>1.846705488156557</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1.821057394850547</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.969688637793288</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2.0847582646007</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.545478633832395</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.784249300589771</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1.720377123512736</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.81339345193167</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1.816747050579617</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1.473731204441798</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.456735985703921</v>
+      </c>
+      <c r="M40" t="n">
+        <v/>
+      </c>
+      <c r="N40" t="n">
+        <v>1.817914526353068</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.885136652359405</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1.955219227583847</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.939094815947656</v>
+      </c>
+      <c r="R40" t="n">
+        <v>2.049166954603483</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.7813264556246253</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1.144154571151934</v>
+      </c>
+      <c r="U40" t="n">
+        <v>1.782469157027053</v>
+      </c>
+      <c r="V40" t="n">
+        <v>1.771676589262436</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>JS</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2.19814521384585</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2.085334997103887</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2.160546643109491</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2.187416481221013</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2.136791669123135</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1.970475738144349</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.100006419519111</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2.187832350559419</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1.737880091003279</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1.712799317709126</v>
+      </c>
+      <c r="M41" t="n">
+        <v/>
+      </c>
+      <c r="N41" t="n">
+        <v>2.649233137387162</v>
+      </c>
+      <c r="O41" t="n">
+        <v>2.585547778036334</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2.264863084577176</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2.253521495185312</v>
+      </c>
+      <c r="R41" t="n">
+        <v>2.318268421862938</v>
+      </c>
+      <c r="S41" t="n">
+        <v>2.248919358016478</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.800002722742227</v>
+      </c>
+      <c r="U41" t="n">
+        <v>2.534947964165799</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2.47279176907465</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AOr</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1.465421851650792</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.616907326787175</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1.808251288231164</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.244711436227292</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1.884176190176511</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.35349798089488</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1.745016194476912</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2.014585903728875</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1.639405019942544</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1.720214228741179</v>
+      </c>
+      <c r="M42" t="n">
+        <v/>
+      </c>
+      <c r="N42" t="n">
+        <v>2.117538337688619</v>
+      </c>
+      <c r="O42" t="n">
+        <v>2.046625884628753</v>
+      </c>
+      <c r="P42" t="n">
+        <v>1.984729003288086</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1.960694713853754</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1.979620480213499</v>
+      </c>
+      <c r="S42" t="n">
+        <v>1.391961733344009</v>
+      </c>
+      <c r="T42" t="n">
+        <v>1.495987152055055</v>
+      </c>
+      <c r="U42" t="n">
+        <v>1.984760279882844</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2.032504434828468</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2.095769434592255</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2.05832670262809</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.230203730664122</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2.151497294532881</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2.265325167624174</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.873414544713265</v>
+      </c>
+      <c r="I43" t="n">
+        <v>2.128219583947527</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2.480833285913028</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2.154534833035016</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.157603029028635</v>
+      </c>
+      <c r="M43" t="n">
+        <v/>
+      </c>
+      <c r="N43" t="n">
+        <v>2.349606994239055</v>
+      </c>
+      <c r="O43" t="n">
+        <v>2.273370738858302</v>
+      </c>
+      <c r="P43" t="n">
+        <v>2.174999225154675</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1.999691713858884</v>
+      </c>
+      <c r="R43" t="n">
+        <v>2.254805203058166</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1.712935565692674</v>
+      </c>
+      <c r="T43" t="n">
+        <v>1.359428272584472</v>
+      </c>
+      <c r="U43" t="n">
+        <v>2.218728247764188</v>
+      </c>
+      <c r="V43" t="n">
+        <v>1.445260231071668</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CG</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1.529083700725893</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1.884645511633816</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.105299702893814</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.440300825018261</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1.894255236319918</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1.475541076353048</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.59632243606325</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1.807161239563339</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1.027421090875456</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.73117848603783</v>
+      </c>
+      <c r="M44" t="n">
+        <v/>
+      </c>
+      <c r="N44" t="n">
+        <v>1.822688469375817</v>
+      </c>
+      <c r="O44" t="n">
+        <v>2.257410057374006</v>
+      </c>
+      <c r="P44" t="n">
+        <v>2.09595835623572</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>2.183991941689351</v>
+      </c>
+      <c r="R44" t="n">
+        <v>2.264309405730935</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1.324428760137135</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1.220804811874782</v>
+      </c>
+      <c r="U44" t="n">
+        <v>1.855715479132856</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2.116704145020841</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1.761715947008601</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1.548073494304787</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.638514927761295</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.887253819697695</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1.57616976087278</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.756733338871027</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1.342733220901325</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1.953765677312807</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1.747115550286415</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1.732687612223945</v>
+      </c>
+      <c r="M45" t="n">
+        <v/>
+      </c>
+      <c r="N45" t="n">
+        <v>1.627297250599028</v>
+      </c>
+      <c r="O45" t="n">
+        <v>1.757363011717612</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1.711799545312622</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1.678963792605864</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1.745596644484272</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1.407320489130472</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.7673581093452568</v>
+      </c>
+      <c r="U45" t="n">
+        <v>1.806226766875661</v>
+      </c>
+      <c r="V45" t="n">
+        <v>1.58116899147504</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.336958315103918</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1.273577282787253</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.816679060932044</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1.197024200900441</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1.500919503914353</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1.359795884940916</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.286479683608428</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1.673067810383043</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1.789283037586396</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1.799491456328317</v>
+      </c>
+      <c r="M46" t="n">
+        <v/>
+      </c>
+      <c r="N46" t="n">
+        <v>2.153017788117499</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2.29033600381467</v>
+      </c>
+      <c r="P46" t="n">
+        <v>1.892843116432654</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1.798951371872497</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1.933242677062141</v>
+      </c>
+      <c r="S46" t="n">
+        <v>1.306532312128597</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1.361234078727617</v>
+      </c>
+      <c r="U46" t="n">
+        <v>2.125514491565056</v>
+      </c>
+      <c r="V46" t="n">
+        <v>1.915704030905858</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MiM</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2.141094703661915</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.263789305839658</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2.300451609758958</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2.154011104533201</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2.200216808471293</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2.219373219100706</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2.149831497677346</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2.364896837141451</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1.798439239026421</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1.803733883225656</v>
+      </c>
+      <c r="M47" t="n">
+        <v/>
+      </c>
+      <c r="N47" t="n">
+        <v>2.496621163120712</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.655844014060665</v>
+      </c>
+      <c r="P47" t="n">
+        <v>2.415024808330931</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2.388711785792675</v>
+      </c>
+      <c r="R47" t="n">
+        <v>2.49959167821896</v>
+      </c>
+      <c r="S47" t="n">
+        <v>2.078610757907007</v>
+      </c>
+      <c r="T47" t="n">
+        <v>1.942871243585486</v>
+      </c>
+      <c r="U47" t="n">
+        <v>2.367168137989498</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2.463844838478356</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>JaM</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2.406987346362906</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.36854610894488</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.270307744984759</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2.313338549114736</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2.424027700144207</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2.257477011010904</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2.254344746994005</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2.397762470287671</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.843955519632756</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.083721216742153</v>
+      </c>
+      <c r="M48" t="n">
+        <v/>
+      </c>
+      <c r="N48" t="n">
+        <v>2.407794718404622</v>
+      </c>
+      <c r="O48" t="n">
+        <v>2.47301078625571</v>
+      </c>
+      <c r="P48" t="n">
+        <v>2.386484836645799</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.217568012833066</v>
+      </c>
+      <c r="R48" t="n">
+        <v>2.328800507750075</v>
+      </c>
+      <c r="S48" t="n">
+        <v>2.349691741807787</v>
+      </c>
+      <c r="T48" t="n">
+        <v>2.509222291879965</v>
+      </c>
+      <c r="U48" t="n">
+        <v>2.387054252834779</v>
+      </c>
+      <c r="V48" t="n">
+        <v>2.486064947884257</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Average: Typically Developing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Subset</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1.911351507018986</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.931497755129457</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2.075845210588148</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1.859540113606328</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.972744393382454</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1.829148492080869</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.833916380080333</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2.085258340217547</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.696545070735942</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1.809743873374948</v>
+      </c>
+      <c r="M49" t="n">
+        <v/>
+      </c>
+      <c r="N49" t="n">
+        <v>2.16552175594962</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2.272252380309588</v>
+      </c>
+      <c r="P49" t="n">
+        <v>2.112149025034178</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2.057561866223163</v>
+      </c>
+      <c r="R49" t="n">
+        <v>2.174222686596371</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.651220680055597</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1.513134512736467</v>
+      </c>
+      <c r="U49" t="n">
+        <v>2.134728062169361</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2.031651942896638</v>
       </c>
     </row>
   </sheetData>
@@ -3291,7 +4011,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4138,64 +4858,64 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.057093547330473</v>
+        <v>2.024668147718512</v>
       </c>
       <c r="D12" t="n">
-        <v>1.959760537708682</v>
+        <v>1.96868605083528</v>
       </c>
       <c r="E12" t="n">
-        <v>2.018522577006388</v>
+        <v>1.997235502033564</v>
       </c>
       <c r="F12" t="n">
-        <v>1.843825449929359</v>
+        <v>1.890965750974551</v>
       </c>
       <c r="G12" t="n">
-        <v>1.986383989072011</v>
+        <v>1.973309945131826</v>
       </c>
       <c r="H12" t="n">
-        <v>1.979454547823752</v>
+        <v>2.025951767250887</v>
       </c>
       <c r="I12" t="n">
-        <v>1.757312822854038</v>
+        <v>1.834479080590469</v>
       </c>
       <c r="J12" t="n">
-        <v>2.145466290143831</v>
+        <v>2.175618676112611</v>
       </c>
       <c r="K12" t="n">
-        <v>1.929526700683982</v>
+        <v>1.991936647761554</v>
       </c>
       <c r="L12" t="n">
-        <v>1.821971139194069</v>
+        <v>1.836382690079349</v>
       </c>
       <c r="M12" t="n">
         <v>1.995904382483224</v>
       </c>
       <c r="N12" t="n">
-        <v>2.369037164018575</v>
+        <v>2.348177949782953</v>
       </c>
       <c r="O12" t="n">
-        <v>2.448812293885807</v>
+        <v>2.415581819369827</v>
       </c>
       <c r="P12" t="n">
-        <v>2.211831315665458</v>
+        <v>2.222630520845329</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.085934481024001</v>
+        <v>2.104067893024136</v>
       </c>
       <c r="R12" t="n">
-        <v>2.138946561132661</v>
+        <v>2.103428264261743</v>
       </c>
       <c r="S12" t="n">
-        <v>1.672039069492139</v>
+        <v>1.694906160218784</v>
       </c>
       <c r="T12" t="n">
-        <v>1.441563175449537</v>
+        <v>1.566122955680536</v>
       </c>
       <c r="U12" t="n">
-        <v>2.327030767708496</v>
+        <v>2.33547336142582</v>
       </c>
       <c r="V12" t="n">
-        <v>2.137540924940734</v>
+        <v>2.160336426143453</v>
       </c>
     </row>
     <row r="13">
@@ -6140,6 +6860,726 @@
       </c>
       <c r="V39" t="n">
         <v>1.846705488156557</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1.821057394850547</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.969688637793288</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2.0847582646007</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.545478633832395</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.784249300589771</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1.720377123512736</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.81339345193167</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1.816747050579617</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1.473731204441798</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.456735985703921</v>
+      </c>
+      <c r="M40" t="n">
+        <v/>
+      </c>
+      <c r="N40" t="n">
+        <v>1.817914526353068</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.885136652359405</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1.955219227583847</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.939094815947656</v>
+      </c>
+      <c r="R40" t="n">
+        <v>2.049166954603483</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.7813264556246253</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1.144154571151934</v>
+      </c>
+      <c r="U40" t="n">
+        <v>1.782469157027053</v>
+      </c>
+      <c r="V40" t="n">
+        <v>1.771676589262436</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>JS</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2.19814521384585</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2.085334997103887</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2.160546643109491</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2.187416481221013</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2.136791669123135</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1.970475738144349</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.100006419519111</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2.187832350559419</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1.737880091003279</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1.712799317709126</v>
+      </c>
+      <c r="M41" t="n">
+        <v/>
+      </c>
+      <c r="N41" t="n">
+        <v>2.649233137387162</v>
+      </c>
+      <c r="O41" t="n">
+        <v>2.585547778036334</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2.264863084577176</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2.253521495185312</v>
+      </c>
+      <c r="R41" t="n">
+        <v>2.318268421862938</v>
+      </c>
+      <c r="S41" t="n">
+        <v>2.248919358016478</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.800002722742227</v>
+      </c>
+      <c r="U41" t="n">
+        <v>2.534947964165799</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2.47279176907465</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AOr</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1.465421851650792</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.616907326787175</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1.808251288231164</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.244711436227292</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1.884176190176511</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.35349798089488</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1.745016194476912</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2.014585903728875</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1.639405019942544</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1.720214228741179</v>
+      </c>
+      <c r="M42" t="n">
+        <v/>
+      </c>
+      <c r="N42" t="n">
+        <v>2.117538337688619</v>
+      </c>
+      <c r="O42" t="n">
+        <v>2.046625884628753</v>
+      </c>
+      <c r="P42" t="n">
+        <v>1.984729003288086</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1.960694713853754</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1.979620480213499</v>
+      </c>
+      <c r="S42" t="n">
+        <v>1.391961733344009</v>
+      </c>
+      <c r="T42" t="n">
+        <v>1.495987152055055</v>
+      </c>
+      <c r="U42" t="n">
+        <v>1.984760279882844</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2.032504434828468</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2.095769434592255</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2.05832670262809</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.230203730664122</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2.151497294532881</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2.265325167624174</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.873414544713265</v>
+      </c>
+      <c r="I43" t="n">
+        <v>2.128219583947527</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2.480833285913028</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2.154534833035016</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.157603029028635</v>
+      </c>
+      <c r="M43" t="n">
+        <v/>
+      </c>
+      <c r="N43" t="n">
+        <v>2.349606994239055</v>
+      </c>
+      <c r="O43" t="n">
+        <v>2.273370738858302</v>
+      </c>
+      <c r="P43" t="n">
+        <v>2.174999225154675</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1.999691713858884</v>
+      </c>
+      <c r="R43" t="n">
+        <v>2.254805203058166</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1.712935565692674</v>
+      </c>
+      <c r="T43" t="n">
+        <v>1.359428272584472</v>
+      </c>
+      <c r="U43" t="n">
+        <v>2.218728247764188</v>
+      </c>
+      <c r="V43" t="n">
+        <v>1.445260231071668</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CG</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1.529083700725893</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1.884645511633816</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.105299702893814</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.440300825018261</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1.894255236319918</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1.475541076353048</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.59632243606325</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1.807161239563339</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1.027421090875456</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.73117848603783</v>
+      </c>
+      <c r="M44" t="n">
+        <v/>
+      </c>
+      <c r="N44" t="n">
+        <v>1.822688469375817</v>
+      </c>
+      <c r="O44" t="n">
+        <v>2.257410057374006</v>
+      </c>
+      <c r="P44" t="n">
+        <v>2.09595835623572</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>2.183991941689351</v>
+      </c>
+      <c r="R44" t="n">
+        <v>2.264309405730935</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1.324428760137135</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1.220804811874782</v>
+      </c>
+      <c r="U44" t="n">
+        <v>1.855715479132856</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2.116704145020841</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1.761715947008601</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1.548073494304787</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.638514927761295</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.887253819697695</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1.57616976087278</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.756733338871027</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1.342733220901325</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1.953765677312807</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1.747115550286415</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1.732687612223945</v>
+      </c>
+      <c r="M45" t="n">
+        <v/>
+      </c>
+      <c r="N45" t="n">
+        <v>1.627297250599028</v>
+      </c>
+      <c r="O45" t="n">
+        <v>1.757363011717612</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1.711799545312622</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1.678963792605864</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1.745596644484272</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1.407320489130472</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.7673581093452568</v>
+      </c>
+      <c r="U45" t="n">
+        <v>1.806226766875661</v>
+      </c>
+      <c r="V45" t="n">
+        <v>1.58116899147504</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.336958315103918</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1.273577282787253</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.816679060932044</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1.197024200900441</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1.500919503914353</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1.359795884940916</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.286479683608428</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1.673067810383043</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1.789283037586396</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1.799491456328317</v>
+      </c>
+      <c r="M46" t="n">
+        <v/>
+      </c>
+      <c r="N46" t="n">
+        <v>2.153017788117499</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2.29033600381467</v>
+      </c>
+      <c r="P46" t="n">
+        <v>1.892843116432654</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1.798951371872497</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1.933242677062141</v>
+      </c>
+      <c r="S46" t="n">
+        <v>1.306532312128597</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1.361234078727617</v>
+      </c>
+      <c r="U46" t="n">
+        <v>2.125514491565056</v>
+      </c>
+      <c r="V46" t="n">
+        <v>1.915704030905858</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MiM</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2.141094703661915</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.263789305839658</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2.300451609758958</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2.154011104533201</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2.200216808471293</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2.219373219100706</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2.149831497677346</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2.364896837141451</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1.798439239026421</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1.803733883225656</v>
+      </c>
+      <c r="M47" t="n">
+        <v/>
+      </c>
+      <c r="N47" t="n">
+        <v>2.496621163120712</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.655844014060665</v>
+      </c>
+      <c r="P47" t="n">
+        <v>2.415024808330931</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2.388711785792675</v>
+      </c>
+      <c r="R47" t="n">
+        <v>2.49959167821896</v>
+      </c>
+      <c r="S47" t="n">
+        <v>2.078610757907007</v>
+      </c>
+      <c r="T47" t="n">
+        <v>1.942871243585486</v>
+      </c>
+      <c r="U47" t="n">
+        <v>2.367168137989498</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2.463844838478356</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>JaM</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2.406987346362906</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.36854610894488</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.270307744984759</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2.313338549114736</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2.424027700144207</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2.257477011010904</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2.254344746994005</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2.397762470287671</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.843955519632756</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.083721216742153</v>
+      </c>
+      <c r="M48" t="n">
+        <v/>
+      </c>
+      <c r="N48" t="n">
+        <v>2.407794718404622</v>
+      </c>
+      <c r="O48" t="n">
+        <v>2.47301078625571</v>
+      </c>
+      <c r="P48" t="n">
+        <v>2.386484836645799</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.217568012833066</v>
+      </c>
+      <c r="R48" t="n">
+        <v>2.328800507750075</v>
+      </c>
+      <c r="S48" t="n">
+        <v>2.349691741807787</v>
+      </c>
+      <c r="T48" t="n">
+        <v>2.509222291879965</v>
+      </c>
+      <c r="U48" t="n">
+        <v>2.387054252834779</v>
+      </c>
+      <c r="V48" t="n">
+        <v>2.486064947884257</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Average: Typically Developing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Subset</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1.911351507018986</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.931497755129457</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2.075845210588148</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1.859540113606328</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.972744393382454</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1.829148492080869</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.833916380080333</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2.085258340217547</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.696545070735942</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1.809743873374948</v>
+      </c>
+      <c r="M49" t="n">
+        <v/>
+      </c>
+      <c r="N49" t="n">
+        <v>2.16552175594962</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2.272252380309588</v>
+      </c>
+      <c r="P49" t="n">
+        <v>2.112149025034178</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2.057561866223163</v>
+      </c>
+      <c r="R49" t="n">
+        <v>2.174222686596371</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.651220680055597</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1.513134512736467</v>
+      </c>
+      <c r="U49" t="n">
+        <v>2.134728062169361</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2.031651942896638</v>
       </c>
     </row>
   </sheetData>
@@ -6153,7 +7593,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7000,64 +8440,64 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.057093547330473</v>
+        <v>2.024668147718512</v>
       </c>
       <c r="D12" t="n">
-        <v>1.959760537708682</v>
+        <v>1.96868605083528</v>
       </c>
       <c r="E12" t="n">
-        <v>2.018522577006388</v>
+        <v>1.997235502033564</v>
       </c>
       <c r="F12" t="n">
-        <v>1.843825449929359</v>
+        <v>1.890965750974551</v>
       </c>
       <c r="G12" t="n">
-        <v>1.986383989072011</v>
+        <v>1.973309945131826</v>
       </c>
       <c r="H12" t="n">
-        <v>1.979454547823752</v>
+        <v>2.025951767250887</v>
       </c>
       <c r="I12" t="n">
-        <v>1.757312822854038</v>
+        <v>1.834479080590469</v>
       </c>
       <c r="J12" t="n">
-        <v>2.145466290143831</v>
+        <v>2.175618676112611</v>
       </c>
       <c r="K12" t="n">
-        <v>1.929526700683982</v>
+        <v>1.991936647761554</v>
       </c>
       <c r="L12" t="n">
-        <v>1.821971139194069</v>
+        <v>1.836382690079349</v>
       </c>
       <c r="M12" t="n">
         <v>1.995904382483224</v>
       </c>
       <c r="N12" t="n">
-        <v>2.369037164018575</v>
+        <v>2.348177949782953</v>
       </c>
       <c r="O12" t="n">
-        <v>2.448812293885807</v>
+        <v>2.415581819369827</v>
       </c>
       <c r="P12" t="n">
-        <v>2.211831315665458</v>
+        <v>2.222630520845329</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.085934481024001</v>
+        <v>2.104067893024136</v>
       </c>
       <c r="R12" t="n">
-        <v>2.138946561132661</v>
+        <v>2.103428264261743</v>
       </c>
       <c r="S12" t="n">
-        <v>1.672039069492139</v>
+        <v>1.694906160218784</v>
       </c>
       <c r="T12" t="n">
-        <v>1.441563175449537</v>
+        <v>1.566122955680536</v>
       </c>
       <c r="U12" t="n">
-        <v>2.327030767708496</v>
+        <v>2.33547336142582</v>
       </c>
       <c r="V12" t="n">
-        <v>2.137540924940734</v>
+        <v>2.160336426143453</v>
       </c>
     </row>
     <row r="13">
@@ -9002,6 +10442,726 @@
       </c>
       <c r="V39" t="n">
         <v>1.846705488156557</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1.821057394850547</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.969688637793288</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2.0847582646007</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.545478633832395</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.784249300589771</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1.720377123512736</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.81339345193167</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1.816747050579617</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1.473731204441798</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.456735985703921</v>
+      </c>
+      <c r="M40" t="n">
+        <v/>
+      </c>
+      <c r="N40" t="n">
+        <v>1.817914526353068</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.885136652359405</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1.955219227583847</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.939094815947656</v>
+      </c>
+      <c r="R40" t="n">
+        <v>2.049166954603483</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.7813264556246253</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1.144154571151934</v>
+      </c>
+      <c r="U40" t="n">
+        <v>1.782469157027053</v>
+      </c>
+      <c r="V40" t="n">
+        <v>1.771676589262436</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>JS</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2.19814521384585</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2.085334997103887</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2.160546643109491</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2.187416481221013</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2.136791669123135</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1.970475738144349</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.100006419519111</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2.187832350559419</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1.737880091003279</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1.712799317709126</v>
+      </c>
+      <c r="M41" t="n">
+        <v/>
+      </c>
+      <c r="N41" t="n">
+        <v>2.649233137387162</v>
+      </c>
+      <c r="O41" t="n">
+        <v>2.585547778036334</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2.264863084577176</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2.253521495185312</v>
+      </c>
+      <c r="R41" t="n">
+        <v>2.318268421862938</v>
+      </c>
+      <c r="S41" t="n">
+        <v>2.248919358016478</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.800002722742227</v>
+      </c>
+      <c r="U41" t="n">
+        <v>2.534947964165799</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2.47279176907465</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AOr</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1.465421851650792</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.616907326787175</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1.808251288231164</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.244711436227292</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1.884176190176511</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.35349798089488</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1.745016194476912</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2.014585903728875</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1.639405019942544</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1.720214228741179</v>
+      </c>
+      <c r="M42" t="n">
+        <v/>
+      </c>
+      <c r="N42" t="n">
+        <v>2.117538337688619</v>
+      </c>
+      <c r="O42" t="n">
+        <v>2.046625884628753</v>
+      </c>
+      <c r="P42" t="n">
+        <v>1.984729003288086</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1.960694713853754</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1.979620480213499</v>
+      </c>
+      <c r="S42" t="n">
+        <v>1.391961733344009</v>
+      </c>
+      <c r="T42" t="n">
+        <v>1.495987152055055</v>
+      </c>
+      <c r="U42" t="n">
+        <v>1.984760279882844</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2.032504434828468</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2.095769434592255</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2.05832670262809</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.230203730664122</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2.151497294532881</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2.265325167624174</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.873414544713265</v>
+      </c>
+      <c r="I43" t="n">
+        <v>2.128219583947527</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2.480833285913028</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2.154534833035016</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.157603029028635</v>
+      </c>
+      <c r="M43" t="n">
+        <v/>
+      </c>
+      <c r="N43" t="n">
+        <v>2.349606994239055</v>
+      </c>
+      <c r="O43" t="n">
+        <v>2.273370738858302</v>
+      </c>
+      <c r="P43" t="n">
+        <v>2.174999225154675</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1.999691713858884</v>
+      </c>
+      <c r="R43" t="n">
+        <v>2.254805203058166</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1.712935565692674</v>
+      </c>
+      <c r="T43" t="n">
+        <v>1.359428272584472</v>
+      </c>
+      <c r="U43" t="n">
+        <v>2.218728247764188</v>
+      </c>
+      <c r="V43" t="n">
+        <v>1.445260231071668</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CG</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1.529083700725893</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1.884645511633816</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.105299702893814</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.440300825018261</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1.894255236319918</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1.475541076353048</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.59632243606325</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1.807161239563339</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1.027421090875456</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.73117848603783</v>
+      </c>
+      <c r="M44" t="n">
+        <v/>
+      </c>
+      <c r="N44" t="n">
+        <v>1.822688469375817</v>
+      </c>
+      <c r="O44" t="n">
+        <v>2.257410057374006</v>
+      </c>
+      <c r="P44" t="n">
+        <v>2.09595835623572</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>2.183991941689351</v>
+      </c>
+      <c r="R44" t="n">
+        <v>2.264309405730935</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1.324428760137135</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1.220804811874782</v>
+      </c>
+      <c r="U44" t="n">
+        <v>1.855715479132856</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2.116704145020841</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1.761715947008601</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1.548073494304787</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.638514927761295</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.887253819697695</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1.57616976087278</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.756733338871027</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1.342733220901325</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1.953765677312807</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1.747115550286415</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1.732687612223945</v>
+      </c>
+      <c r="M45" t="n">
+        <v/>
+      </c>
+      <c r="N45" t="n">
+        <v>1.627297250599028</v>
+      </c>
+      <c r="O45" t="n">
+        <v>1.757363011717612</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1.711799545312622</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1.678963792605864</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1.745596644484272</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1.407320489130472</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.7673581093452568</v>
+      </c>
+      <c r="U45" t="n">
+        <v>1.806226766875661</v>
+      </c>
+      <c r="V45" t="n">
+        <v>1.58116899147504</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.336958315103918</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1.273577282787253</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.816679060932044</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1.197024200900441</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1.500919503914353</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1.359795884940916</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.286479683608428</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1.673067810383043</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1.789283037586396</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1.799491456328317</v>
+      </c>
+      <c r="M46" t="n">
+        <v/>
+      </c>
+      <c r="N46" t="n">
+        <v>2.153017788117499</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2.29033600381467</v>
+      </c>
+      <c r="P46" t="n">
+        <v>1.892843116432654</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1.798951371872497</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1.933242677062141</v>
+      </c>
+      <c r="S46" t="n">
+        <v>1.306532312128597</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1.361234078727617</v>
+      </c>
+      <c r="U46" t="n">
+        <v>2.125514491565056</v>
+      </c>
+      <c r="V46" t="n">
+        <v>1.915704030905858</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MiM</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2.141094703661915</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.263789305839658</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2.300451609758958</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2.154011104533201</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2.200216808471293</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2.219373219100706</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2.149831497677346</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2.364896837141451</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1.798439239026421</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1.803733883225656</v>
+      </c>
+      <c r="M47" t="n">
+        <v/>
+      </c>
+      <c r="N47" t="n">
+        <v>2.496621163120712</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.655844014060665</v>
+      </c>
+      <c r="P47" t="n">
+        <v>2.415024808330931</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2.388711785792675</v>
+      </c>
+      <c r="R47" t="n">
+        <v>2.49959167821896</v>
+      </c>
+      <c r="S47" t="n">
+        <v>2.078610757907007</v>
+      </c>
+      <c r="T47" t="n">
+        <v>1.942871243585486</v>
+      </c>
+      <c r="U47" t="n">
+        <v>2.367168137989498</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2.463844838478356</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>JaM</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2.406987346362906</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.36854610894488</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.270307744984759</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2.313338549114736</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2.424027700144207</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2.257477011010904</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2.254344746994005</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2.397762470287671</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.843955519632756</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.083721216742153</v>
+      </c>
+      <c r="M48" t="n">
+        <v/>
+      </c>
+      <c r="N48" t="n">
+        <v>2.407794718404622</v>
+      </c>
+      <c r="O48" t="n">
+        <v>2.47301078625571</v>
+      </c>
+      <c r="P48" t="n">
+        <v>2.386484836645799</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.217568012833066</v>
+      </c>
+      <c r="R48" t="n">
+        <v>2.328800507750075</v>
+      </c>
+      <c r="S48" t="n">
+        <v>2.349691741807787</v>
+      </c>
+      <c r="T48" t="n">
+        <v>2.509222291879965</v>
+      </c>
+      <c r="U48" t="n">
+        <v>2.387054252834779</v>
+      </c>
+      <c r="V48" t="n">
+        <v>2.486064947884257</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Average: Typically Developing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Subset</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1.911351507018986</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.931497755129457</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2.075845210588148</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1.859540113606328</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.972744393382454</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1.829148492080869</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.833916380080333</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2.085258340217547</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.696545070735942</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1.809743873374948</v>
+      </c>
+      <c r="M49" t="n">
+        <v/>
+      </c>
+      <c r="N49" t="n">
+        <v>2.16552175594962</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2.272252380309588</v>
+      </c>
+      <c r="P49" t="n">
+        <v>2.112149025034178</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2.057561866223163</v>
+      </c>
+      <c r="R49" t="n">
+        <v>2.174222686596371</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.651220680055597</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1.513134512736467</v>
+      </c>
+      <c r="U49" t="n">
+        <v>2.134728062169361</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2.031651942896638</v>
       </c>
     </row>
   </sheetData>
@@ -9015,7 +11175,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9862,64 +12022,64 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.057093547330473</v>
+        <v>2.024668147718512</v>
       </c>
       <c r="D12" t="n">
-        <v>1.959760537708682</v>
+        <v>1.96868605083528</v>
       </c>
       <c r="E12" t="n">
-        <v>2.018522577006388</v>
+        <v>1.997235502033564</v>
       </c>
       <c r="F12" t="n">
-        <v>1.843825449929359</v>
+        <v>1.890965750974551</v>
       </c>
       <c r="G12" t="n">
-        <v>1.986383989072011</v>
+        <v>1.973309945131826</v>
       </c>
       <c r="H12" t="n">
-        <v>1.979454547823752</v>
+        <v>2.025951767250887</v>
       </c>
       <c r="I12" t="n">
-        <v>1.757312822854038</v>
+        <v>1.834479080590469</v>
       </c>
       <c r="J12" t="n">
-        <v>2.145466290143831</v>
+        <v>2.175618676112611</v>
       </c>
       <c r="K12" t="n">
-        <v>1.929526700683982</v>
+        <v>1.991936647761554</v>
       </c>
       <c r="L12" t="n">
-        <v>1.821971139194069</v>
+        <v>1.836382690079349</v>
       </c>
       <c r="M12" t="n">
         <v>1.995904382483224</v>
       </c>
       <c r="N12" t="n">
-        <v>2.369037164018575</v>
+        <v>2.348177949782953</v>
       </c>
       <c r="O12" t="n">
-        <v>2.448812293885807</v>
+        <v>2.415581819369827</v>
       </c>
       <c r="P12" t="n">
-        <v>2.211831315665458</v>
+        <v>2.222630520845329</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.085934481024001</v>
+        <v>2.104067893024136</v>
       </c>
       <c r="R12" t="n">
-        <v>2.138946561132661</v>
+        <v>2.103428264261743</v>
       </c>
       <c r="S12" t="n">
-        <v>1.672039069492139</v>
+        <v>1.694906160218784</v>
       </c>
       <c r="T12" t="n">
-        <v>1.441563175449537</v>
+        <v>1.566122955680536</v>
       </c>
       <c r="U12" t="n">
-        <v>2.327030767708496</v>
+        <v>2.33547336142582</v>
       </c>
       <c r="V12" t="n">
-        <v>2.137540924940734</v>
+        <v>2.160336426143453</v>
       </c>
     </row>
     <row r="13">
@@ -11864,6 +14024,726 @@
       </c>
       <c r="V39" t="n">
         <v>1.846705488156557</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1.821057394850547</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.969688637793288</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2.0847582646007</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.545478633832395</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.784249300589771</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1.720377123512736</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.81339345193167</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1.816747050579617</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1.473731204441798</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.456735985703921</v>
+      </c>
+      <c r="M40" t="n">
+        <v/>
+      </c>
+      <c r="N40" t="n">
+        <v>1.817914526353068</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.885136652359405</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1.955219227583847</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.939094815947656</v>
+      </c>
+      <c r="R40" t="n">
+        <v>2.049166954603483</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.7813264556246253</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1.144154571151934</v>
+      </c>
+      <c r="U40" t="n">
+        <v>1.782469157027053</v>
+      </c>
+      <c r="V40" t="n">
+        <v>1.771676589262436</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>JS</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2.19814521384585</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2.085334997103887</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2.160546643109491</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2.187416481221013</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2.136791669123135</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1.970475738144349</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.100006419519111</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2.187832350559419</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1.737880091003279</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1.712799317709126</v>
+      </c>
+      <c r="M41" t="n">
+        <v/>
+      </c>
+      <c r="N41" t="n">
+        <v>2.649233137387162</v>
+      </c>
+      <c r="O41" t="n">
+        <v>2.585547778036334</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2.264863084577176</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2.253521495185312</v>
+      </c>
+      <c r="R41" t="n">
+        <v>2.318268421862938</v>
+      </c>
+      <c r="S41" t="n">
+        <v>2.248919358016478</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.800002722742227</v>
+      </c>
+      <c r="U41" t="n">
+        <v>2.534947964165799</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2.47279176907465</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AOr</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1.465421851650792</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.616907326787175</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1.808251288231164</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.244711436227292</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1.884176190176511</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.35349798089488</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1.745016194476912</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2.014585903728875</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1.639405019942544</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1.720214228741179</v>
+      </c>
+      <c r="M42" t="n">
+        <v/>
+      </c>
+      <c r="N42" t="n">
+        <v>2.117538337688619</v>
+      </c>
+      <c r="O42" t="n">
+        <v>2.046625884628753</v>
+      </c>
+      <c r="P42" t="n">
+        <v>1.984729003288086</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1.960694713853754</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1.979620480213499</v>
+      </c>
+      <c r="S42" t="n">
+        <v>1.391961733344009</v>
+      </c>
+      <c r="T42" t="n">
+        <v>1.495987152055055</v>
+      </c>
+      <c r="U42" t="n">
+        <v>1.984760279882844</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2.032504434828468</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2.095769434592255</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2.05832670262809</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.230203730664122</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2.151497294532881</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2.265325167624174</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.873414544713265</v>
+      </c>
+      <c r="I43" t="n">
+        <v>2.128219583947527</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2.480833285913028</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2.154534833035016</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.157603029028635</v>
+      </c>
+      <c r="M43" t="n">
+        <v/>
+      </c>
+      <c r="N43" t="n">
+        <v>2.349606994239055</v>
+      </c>
+      <c r="O43" t="n">
+        <v>2.273370738858302</v>
+      </c>
+      <c r="P43" t="n">
+        <v>2.174999225154675</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1.999691713858884</v>
+      </c>
+      <c r="R43" t="n">
+        <v>2.254805203058166</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1.712935565692674</v>
+      </c>
+      <c r="T43" t="n">
+        <v>1.359428272584472</v>
+      </c>
+      <c r="U43" t="n">
+        <v>2.218728247764188</v>
+      </c>
+      <c r="V43" t="n">
+        <v>1.445260231071668</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CG</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1.529083700725893</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1.884645511633816</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.105299702893814</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.440300825018261</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1.894255236319918</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1.475541076353048</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.59632243606325</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1.807161239563339</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1.027421090875456</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.73117848603783</v>
+      </c>
+      <c r="M44" t="n">
+        <v/>
+      </c>
+      <c r="N44" t="n">
+        <v>1.822688469375817</v>
+      </c>
+      <c r="O44" t="n">
+        <v>2.257410057374006</v>
+      </c>
+      <c r="P44" t="n">
+        <v>2.09595835623572</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>2.183991941689351</v>
+      </c>
+      <c r="R44" t="n">
+        <v>2.264309405730935</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1.324428760137135</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1.220804811874782</v>
+      </c>
+      <c r="U44" t="n">
+        <v>1.855715479132856</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2.116704145020841</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1.761715947008601</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1.548073494304787</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.638514927761295</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.887253819697695</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1.57616976087278</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.756733338871027</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1.342733220901325</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1.953765677312807</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1.747115550286415</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1.732687612223945</v>
+      </c>
+      <c r="M45" t="n">
+        <v/>
+      </c>
+      <c r="N45" t="n">
+        <v>1.627297250599028</v>
+      </c>
+      <c r="O45" t="n">
+        <v>1.757363011717612</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1.711799545312622</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1.678963792605864</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1.745596644484272</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1.407320489130472</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.7673581093452568</v>
+      </c>
+      <c r="U45" t="n">
+        <v>1.806226766875661</v>
+      </c>
+      <c r="V45" t="n">
+        <v>1.58116899147504</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.336958315103918</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1.273577282787253</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.816679060932044</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1.197024200900441</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1.500919503914353</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1.359795884940916</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.286479683608428</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1.673067810383043</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1.789283037586396</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1.799491456328317</v>
+      </c>
+      <c r="M46" t="n">
+        <v/>
+      </c>
+      <c r="N46" t="n">
+        <v>2.153017788117499</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2.29033600381467</v>
+      </c>
+      <c r="P46" t="n">
+        <v>1.892843116432654</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1.798951371872497</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1.933242677062141</v>
+      </c>
+      <c r="S46" t="n">
+        <v>1.306532312128597</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1.361234078727617</v>
+      </c>
+      <c r="U46" t="n">
+        <v>2.125514491565056</v>
+      </c>
+      <c r="V46" t="n">
+        <v>1.915704030905858</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MiM</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2.141094703661915</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.263789305839658</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2.300451609758958</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2.154011104533201</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2.200216808471293</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2.219373219100706</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2.149831497677346</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2.364896837141451</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1.798439239026421</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1.803733883225656</v>
+      </c>
+      <c r="M47" t="n">
+        <v/>
+      </c>
+      <c r="N47" t="n">
+        <v>2.496621163120712</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.655844014060665</v>
+      </c>
+      <c r="P47" t="n">
+        <v>2.415024808330931</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2.388711785792675</v>
+      </c>
+      <c r="R47" t="n">
+        <v>2.49959167821896</v>
+      </c>
+      <c r="S47" t="n">
+        <v>2.078610757907007</v>
+      </c>
+      <c r="T47" t="n">
+        <v>1.942871243585486</v>
+      </c>
+      <c r="U47" t="n">
+        <v>2.367168137989498</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2.463844838478356</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>JaM</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2.406987346362906</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.36854610894488</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.270307744984759</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2.313338549114736</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2.424027700144207</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2.257477011010904</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2.254344746994005</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2.397762470287671</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.843955519632756</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.083721216742153</v>
+      </c>
+      <c r="M48" t="n">
+        <v/>
+      </c>
+      <c r="N48" t="n">
+        <v>2.407794718404622</v>
+      </c>
+      <c r="O48" t="n">
+        <v>2.47301078625571</v>
+      </c>
+      <c r="P48" t="n">
+        <v>2.386484836645799</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.217568012833066</v>
+      </c>
+      <c r="R48" t="n">
+        <v>2.328800507750075</v>
+      </c>
+      <c r="S48" t="n">
+        <v>2.349691741807787</v>
+      </c>
+      <c r="T48" t="n">
+        <v>2.509222291879965</v>
+      </c>
+      <c r="U48" t="n">
+        <v>2.387054252834779</v>
+      </c>
+      <c r="V48" t="n">
+        <v>2.486064947884257</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Average: Typically Developing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Subset</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1.911351507018986</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.931497755129457</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2.075845210588148</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1.859540113606328</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.972744393382454</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1.829148492080869</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.833916380080333</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2.085258340217547</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.696545070735942</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1.809743873374948</v>
+      </c>
+      <c r="M49" t="n">
+        <v/>
+      </c>
+      <c r="N49" t="n">
+        <v>2.16552175594962</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2.272252380309588</v>
+      </c>
+      <c r="P49" t="n">
+        <v>2.112149025034178</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2.057561866223163</v>
+      </c>
+      <c r="R49" t="n">
+        <v>2.174222686596371</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.651220680055597</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1.513134512736467</v>
+      </c>
+      <c r="U49" t="n">
+        <v>2.134728062169361</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2.031651942896638</v>
       </c>
     </row>
   </sheetData>
@@ -11877,7 +14757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -12724,64 +15604,64 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>2.057093547330473</v>
+        <v>2.024668147718512</v>
       </c>
       <c r="D12" t="n">
-        <v>1.959760537708682</v>
+        <v>1.96868605083528</v>
       </c>
       <c r="E12" t="n">
-        <v>2.018522577006388</v>
+        <v>1.997235502033564</v>
       </c>
       <c r="F12" t="n">
-        <v>1.843825449929359</v>
+        <v>1.890965750974551</v>
       </c>
       <c r="G12" t="n">
-        <v>1.986383989072011</v>
+        <v>1.973309945131826</v>
       </c>
       <c r="H12" t="n">
-        <v>1.979454547823752</v>
+        <v>2.025951767250887</v>
       </c>
       <c r="I12" t="n">
-        <v>1.757312822854038</v>
+        <v>1.834479080590469</v>
       </c>
       <c r="J12" t="n">
-        <v>2.145466290143831</v>
+        <v>2.175618676112611</v>
       </c>
       <c r="K12" t="n">
-        <v>1.929526700683982</v>
+        <v>1.991936647761554</v>
       </c>
       <c r="L12" t="n">
-        <v>1.821971139194069</v>
+        <v>1.836382690079349</v>
       </c>
       <c r="M12" t="n">
         <v>1.995904382483224</v>
       </c>
       <c r="N12" t="n">
-        <v>2.369037164018575</v>
+        <v>2.348177949782953</v>
       </c>
       <c r="O12" t="n">
-        <v>2.448812293885807</v>
+        <v>2.415581819369827</v>
       </c>
       <c r="P12" t="n">
-        <v>2.211831315665458</v>
+        <v>2.222630520845329</v>
       </c>
       <c r="Q12" t="n">
-        <v>2.085934481024001</v>
+        <v>2.104067893024136</v>
       </c>
       <c r="R12" t="n">
-        <v>2.138946561132661</v>
+        <v>2.103428264261743</v>
       </c>
       <c r="S12" t="n">
-        <v>1.672039069492139</v>
+        <v>1.694906160218784</v>
       </c>
       <c r="T12" t="n">
-        <v>1.441563175449537</v>
+        <v>1.566122955680536</v>
       </c>
       <c r="U12" t="n">
-        <v>2.327030767708496</v>
+        <v>2.33547336142582</v>
       </c>
       <c r="V12" t="n">
-        <v>2.137540924940734</v>
+        <v>2.160336426143453</v>
       </c>
     </row>
     <row r="13">
@@ -14726,6 +17606,726 @@
       </c>
       <c r="V39" t="n">
         <v>1.846705488156557</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>DD</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1.821057394850547</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.969688637793288</v>
+      </c>
+      <c r="E40" t="n">
+        <v>2.0847582646007</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.545478633832395</v>
+      </c>
+      <c r="G40" t="n">
+        <v>1.784249300589771</v>
+      </c>
+      <c r="H40" t="n">
+        <v>1.720377123512736</v>
+      </c>
+      <c r="I40" t="n">
+        <v>1.81339345193167</v>
+      </c>
+      <c r="J40" t="n">
+        <v>1.816747050579617</v>
+      </c>
+      <c r="K40" t="n">
+        <v>1.473731204441798</v>
+      </c>
+      <c r="L40" t="n">
+        <v>1.456735985703921</v>
+      </c>
+      <c r="M40" t="n">
+        <v/>
+      </c>
+      <c r="N40" t="n">
+        <v>1.817914526353068</v>
+      </c>
+      <c r="O40" t="n">
+        <v>1.885136652359405</v>
+      </c>
+      <c r="P40" t="n">
+        <v>1.955219227583847</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>1.939094815947656</v>
+      </c>
+      <c r="R40" t="n">
+        <v>2.049166954603483</v>
+      </c>
+      <c r="S40" t="n">
+        <v>0.7813264556246253</v>
+      </c>
+      <c r="T40" t="n">
+        <v>1.144154571151934</v>
+      </c>
+      <c r="U40" t="n">
+        <v>1.782469157027053</v>
+      </c>
+      <c r="V40" t="n">
+        <v>1.771676589262436</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>JS</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>2.19814521384585</v>
+      </c>
+      <c r="D41" t="n">
+        <v>2.085334997103887</v>
+      </c>
+      <c r="E41" t="n">
+        <v>2.160546643109491</v>
+      </c>
+      <c r="F41" t="n">
+        <v>2.187416481221013</v>
+      </c>
+      <c r="G41" t="n">
+        <v>2.136791669123135</v>
+      </c>
+      <c r="H41" t="n">
+        <v>1.970475738144349</v>
+      </c>
+      <c r="I41" t="n">
+        <v>2.100006419519111</v>
+      </c>
+      <c r="J41" t="n">
+        <v>2.187832350559419</v>
+      </c>
+      <c r="K41" t="n">
+        <v>1.737880091003279</v>
+      </c>
+      <c r="L41" t="n">
+        <v>1.712799317709126</v>
+      </c>
+      <c r="M41" t="n">
+        <v/>
+      </c>
+      <c r="N41" t="n">
+        <v>2.649233137387162</v>
+      </c>
+      <c r="O41" t="n">
+        <v>2.585547778036334</v>
+      </c>
+      <c r="P41" t="n">
+        <v>2.264863084577176</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>2.253521495185312</v>
+      </c>
+      <c r="R41" t="n">
+        <v>2.318268421862938</v>
+      </c>
+      <c r="S41" t="n">
+        <v>2.248919358016478</v>
+      </c>
+      <c r="T41" t="n">
+        <v>1.800002722742227</v>
+      </c>
+      <c r="U41" t="n">
+        <v>2.534947964165799</v>
+      </c>
+      <c r="V41" t="n">
+        <v>2.47279176907465</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>AOr</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>1.465421851650792</v>
+      </c>
+      <c r="D42" t="n">
+        <v>1.616907326787175</v>
+      </c>
+      <c r="E42" t="n">
+        <v>1.808251288231164</v>
+      </c>
+      <c r="F42" t="n">
+        <v>1.244711436227292</v>
+      </c>
+      <c r="G42" t="n">
+        <v>1.884176190176511</v>
+      </c>
+      <c r="H42" t="n">
+        <v>1.35349798089488</v>
+      </c>
+      <c r="I42" t="n">
+        <v>1.745016194476912</v>
+      </c>
+      <c r="J42" t="n">
+        <v>2.014585903728875</v>
+      </c>
+      <c r="K42" t="n">
+        <v>1.639405019942544</v>
+      </c>
+      <c r="L42" t="n">
+        <v>1.720214228741179</v>
+      </c>
+      <c r="M42" t="n">
+        <v/>
+      </c>
+      <c r="N42" t="n">
+        <v>2.117538337688619</v>
+      </c>
+      <c r="O42" t="n">
+        <v>2.046625884628753</v>
+      </c>
+      <c r="P42" t="n">
+        <v>1.984729003288086</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>1.960694713853754</v>
+      </c>
+      <c r="R42" t="n">
+        <v>1.979620480213499</v>
+      </c>
+      <c r="S42" t="n">
+        <v>1.391961733344009</v>
+      </c>
+      <c r="T42" t="n">
+        <v>1.495987152055055</v>
+      </c>
+      <c r="U42" t="n">
+        <v>1.984760279882844</v>
+      </c>
+      <c r="V42" t="n">
+        <v>2.032504434828468</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>KA</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>2.095769434592255</v>
+      </c>
+      <c r="D43" t="n">
+        <v>2.05832670262809</v>
+      </c>
+      <c r="E43" t="n">
+        <v>2.230203730664122</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2.151497294532881</v>
+      </c>
+      <c r="G43" t="n">
+        <v>2.265325167624174</v>
+      </c>
+      <c r="H43" t="n">
+        <v>1.873414544713265</v>
+      </c>
+      <c r="I43" t="n">
+        <v>2.128219583947527</v>
+      </c>
+      <c r="J43" t="n">
+        <v>2.480833285913028</v>
+      </c>
+      <c r="K43" t="n">
+        <v>2.154534833035016</v>
+      </c>
+      <c r="L43" t="n">
+        <v>2.157603029028635</v>
+      </c>
+      <c r="M43" t="n">
+        <v/>
+      </c>
+      <c r="N43" t="n">
+        <v>2.349606994239055</v>
+      </c>
+      <c r="O43" t="n">
+        <v>2.273370738858302</v>
+      </c>
+      <c r="P43" t="n">
+        <v>2.174999225154675</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>1.999691713858884</v>
+      </c>
+      <c r="R43" t="n">
+        <v>2.254805203058166</v>
+      </c>
+      <c r="S43" t="n">
+        <v>1.712935565692674</v>
+      </c>
+      <c r="T43" t="n">
+        <v>1.359428272584472</v>
+      </c>
+      <c r="U43" t="n">
+        <v>2.218728247764188</v>
+      </c>
+      <c r="V43" t="n">
+        <v>1.445260231071668</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>CG</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>1.529083700725893</v>
+      </c>
+      <c r="D44" t="n">
+        <v>1.884645511633816</v>
+      </c>
+      <c r="E44" t="n">
+        <v>2.105299702893814</v>
+      </c>
+      <c r="F44" t="n">
+        <v>1.440300825018261</v>
+      </c>
+      <c r="G44" t="n">
+        <v>1.894255236319918</v>
+      </c>
+      <c r="H44" t="n">
+        <v>1.475541076353048</v>
+      </c>
+      <c r="I44" t="n">
+        <v>1.59632243606325</v>
+      </c>
+      <c r="J44" t="n">
+        <v>1.807161239563339</v>
+      </c>
+      <c r="K44" t="n">
+        <v>1.027421090875456</v>
+      </c>
+      <c r="L44" t="n">
+        <v>1.73117848603783</v>
+      </c>
+      <c r="M44" t="n">
+        <v/>
+      </c>
+      <c r="N44" t="n">
+        <v>1.822688469375817</v>
+      </c>
+      <c r="O44" t="n">
+        <v>2.257410057374006</v>
+      </c>
+      <c r="P44" t="n">
+        <v>2.09595835623572</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>2.183991941689351</v>
+      </c>
+      <c r="R44" t="n">
+        <v>2.264309405730935</v>
+      </c>
+      <c r="S44" t="n">
+        <v>1.324428760137135</v>
+      </c>
+      <c r="T44" t="n">
+        <v>1.220804811874782</v>
+      </c>
+      <c r="U44" t="n">
+        <v>1.855715479132856</v>
+      </c>
+      <c r="V44" t="n">
+        <v>2.116704145020841</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>BH</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C45" t="n">
+        <v>1.761715947008601</v>
+      </c>
+      <c r="D45" t="n">
+        <v>1.548073494304787</v>
+      </c>
+      <c r="E45" t="n">
+        <v>1.638514927761295</v>
+      </c>
+      <c r="F45" t="n">
+        <v>1.887253819697695</v>
+      </c>
+      <c r="G45" t="n">
+        <v>1.57616976087278</v>
+      </c>
+      <c r="H45" t="n">
+        <v>1.756733338871027</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1.342733220901325</v>
+      </c>
+      <c r="J45" t="n">
+        <v>1.953765677312807</v>
+      </c>
+      <c r="K45" t="n">
+        <v>1.747115550286415</v>
+      </c>
+      <c r="L45" t="n">
+        <v>1.732687612223945</v>
+      </c>
+      <c r="M45" t="n">
+        <v/>
+      </c>
+      <c r="N45" t="n">
+        <v>1.627297250599028</v>
+      </c>
+      <c r="O45" t="n">
+        <v>1.757363011717612</v>
+      </c>
+      <c r="P45" t="n">
+        <v>1.711799545312622</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>1.678963792605864</v>
+      </c>
+      <c r="R45" t="n">
+        <v>1.745596644484272</v>
+      </c>
+      <c r="S45" t="n">
+        <v>1.407320489130472</v>
+      </c>
+      <c r="T45" t="n">
+        <v>0.7673581093452568</v>
+      </c>
+      <c r="U45" t="n">
+        <v>1.806226766875661</v>
+      </c>
+      <c r="V45" t="n">
+        <v>1.58116899147504</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>VH</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C46" t="n">
+        <v>1.336958315103918</v>
+      </c>
+      <c r="D46" t="n">
+        <v>1.273577282787253</v>
+      </c>
+      <c r="E46" t="n">
+        <v>1.816679060932044</v>
+      </c>
+      <c r="F46" t="n">
+        <v>1.197024200900441</v>
+      </c>
+      <c r="G46" t="n">
+        <v>1.500919503914353</v>
+      </c>
+      <c r="H46" t="n">
+        <v>1.359795884940916</v>
+      </c>
+      <c r="I46" t="n">
+        <v>1.286479683608428</v>
+      </c>
+      <c r="J46" t="n">
+        <v>1.673067810383043</v>
+      </c>
+      <c r="K46" t="n">
+        <v>1.789283037586396</v>
+      </c>
+      <c r="L46" t="n">
+        <v>1.799491456328317</v>
+      </c>
+      <c r="M46" t="n">
+        <v/>
+      </c>
+      <c r="N46" t="n">
+        <v>2.153017788117499</v>
+      </c>
+      <c r="O46" t="n">
+        <v>2.29033600381467</v>
+      </c>
+      <c r="P46" t="n">
+        <v>1.892843116432654</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>1.798951371872497</v>
+      </c>
+      <c r="R46" t="n">
+        <v>1.933242677062141</v>
+      </c>
+      <c r="S46" t="n">
+        <v>1.306532312128597</v>
+      </c>
+      <c r="T46" t="n">
+        <v>1.361234078727617</v>
+      </c>
+      <c r="U46" t="n">
+        <v>2.125514491565056</v>
+      </c>
+      <c r="V46" t="n">
+        <v>1.915704030905858</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>MiM</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C47" t="n">
+        <v>2.141094703661915</v>
+      </c>
+      <c r="D47" t="n">
+        <v>2.263789305839658</v>
+      </c>
+      <c r="E47" t="n">
+        <v>2.300451609758958</v>
+      </c>
+      <c r="F47" t="n">
+        <v>2.154011104533201</v>
+      </c>
+      <c r="G47" t="n">
+        <v>2.200216808471293</v>
+      </c>
+      <c r="H47" t="n">
+        <v>2.219373219100706</v>
+      </c>
+      <c r="I47" t="n">
+        <v>2.149831497677346</v>
+      </c>
+      <c r="J47" t="n">
+        <v>2.364896837141451</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1.798439239026421</v>
+      </c>
+      <c r="L47" t="n">
+        <v>1.803733883225656</v>
+      </c>
+      <c r="M47" t="n">
+        <v/>
+      </c>
+      <c r="N47" t="n">
+        <v>2.496621163120712</v>
+      </c>
+      <c r="O47" t="n">
+        <v>2.655844014060665</v>
+      </c>
+      <c r="P47" t="n">
+        <v>2.415024808330931</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>2.388711785792675</v>
+      </c>
+      <c r="R47" t="n">
+        <v>2.49959167821896</v>
+      </c>
+      <c r="S47" t="n">
+        <v>2.078610757907007</v>
+      </c>
+      <c r="T47" t="n">
+        <v>1.942871243585486</v>
+      </c>
+      <c r="U47" t="n">
+        <v>2.367168137989498</v>
+      </c>
+      <c r="V47" t="n">
+        <v>2.463844838478356</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>JaM</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Control</t>
+        </is>
+      </c>
+      <c r="C48" t="n">
+        <v>2.406987346362906</v>
+      </c>
+      <c r="D48" t="n">
+        <v>2.36854610894488</v>
+      </c>
+      <c r="E48" t="n">
+        <v>2.270307744984759</v>
+      </c>
+      <c r="F48" t="n">
+        <v>2.313338549114736</v>
+      </c>
+      <c r="G48" t="n">
+        <v>2.424027700144207</v>
+      </c>
+      <c r="H48" t="n">
+        <v>2.257477011010904</v>
+      </c>
+      <c r="I48" t="n">
+        <v>2.254344746994005</v>
+      </c>
+      <c r="J48" t="n">
+        <v>2.397762470287671</v>
+      </c>
+      <c r="K48" t="n">
+        <v>1.843955519632756</v>
+      </c>
+      <c r="L48" t="n">
+        <v>2.083721216742153</v>
+      </c>
+      <c r="M48" t="n">
+        <v/>
+      </c>
+      <c r="N48" t="n">
+        <v>2.407794718404622</v>
+      </c>
+      <c r="O48" t="n">
+        <v>2.47301078625571</v>
+      </c>
+      <c r="P48" t="n">
+        <v>2.386484836645799</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>2.217568012833066</v>
+      </c>
+      <c r="R48" t="n">
+        <v>2.328800507750075</v>
+      </c>
+      <c r="S48" t="n">
+        <v>2.349691741807787</v>
+      </c>
+      <c r="T48" t="n">
+        <v>2.509222291879965</v>
+      </c>
+      <c r="U48" t="n">
+        <v>2.387054252834779</v>
+      </c>
+      <c r="V48" t="n">
+        <v>2.486064947884257</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Average: Typically Developing</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Subset</t>
+        </is>
+      </c>
+      <c r="C49" t="n">
+        <v>1.911351507018986</v>
+      </c>
+      <c r="D49" t="n">
+        <v>1.931497755129457</v>
+      </c>
+      <c r="E49" t="n">
+        <v>2.075845210588148</v>
+      </c>
+      <c r="F49" t="n">
+        <v>1.859540113606328</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1.972744393382454</v>
+      </c>
+      <c r="H49" t="n">
+        <v>1.829148492080869</v>
+      </c>
+      <c r="I49" t="n">
+        <v>1.833916380080333</v>
+      </c>
+      <c r="J49" t="n">
+        <v>2.085258340217547</v>
+      </c>
+      <c r="K49" t="n">
+        <v>1.696545070735942</v>
+      </c>
+      <c r="L49" t="n">
+        <v>1.809743873374948</v>
+      </c>
+      <c r="M49" t="n">
+        <v/>
+      </c>
+      <c r="N49" t="n">
+        <v>2.16552175594962</v>
+      </c>
+      <c r="O49" t="n">
+        <v>2.272252380309588</v>
+      </c>
+      <c r="P49" t="n">
+        <v>2.112149025034178</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>2.057561866223163</v>
+      </c>
+      <c r="R49" t="n">
+        <v>2.174222686596371</v>
+      </c>
+      <c r="S49" t="n">
+        <v>1.651220680055597</v>
+      </c>
+      <c r="T49" t="n">
+        <v>1.513134512736467</v>
+      </c>
+      <c r="U49" t="n">
+        <v>2.134728062169361</v>
+      </c>
+      <c r="V49" t="n">
+        <v>2.031651942896638</v>
       </c>
     </row>
   </sheetData>

</xml_diff>